<commit_message>
Add average and std
</commit_message>
<xml_diff>
--- a/system_analysis_overview.xlsx
+++ b/system_analysis_overview.xlsx
@@ -28,25 +28,25 @@
     <t>In-In</t>
   </si>
   <si>
+    <t>450249</t>
+  </si>
+  <si>
+    <t>457677</t>
+  </si>
+  <si>
+    <t>1538436</t>
+  </si>
+  <si>
     <t>451623</t>
   </si>
   <si>
+    <t>451606</t>
+  </si>
+  <si>
+    <t>1410412</t>
+  </si>
+  <si>
     <t>1300872</t>
-  </si>
-  <si>
-    <t>1538436</t>
-  </si>
-  <si>
-    <t>457677</t>
-  </si>
-  <si>
-    <t>451606</t>
-  </si>
-  <si>
-    <t>1410412</t>
-  </si>
-  <si>
-    <t>450249</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
Improved comp. speed for finding shortest dists
</commit_message>
<xml_diff>
--- a/system_analysis_overview.xlsx
+++ b/system_analysis_overview.xlsx
@@ -28,25 +28,25 @@
     <t>In-In</t>
   </si>
   <si>
+    <t>1300872</t>
+  </si>
+  <si>
     <t>1410412</t>
   </si>
   <si>
+    <t>457677</t>
+  </si>
+  <si>
+    <t>451623</t>
+  </si>
+  <si>
+    <t>450249</t>
+  </si>
+  <si>
+    <t>1538436</t>
+  </si>
+  <si>
     <t>451606</t>
-  </si>
-  <si>
-    <t>450249</t>
-  </si>
-  <si>
-    <t>1300872</t>
-  </si>
-  <si>
-    <t>1538436</t>
-  </si>
-  <si>
-    <t>451623</t>
-  </si>
-  <si>
-    <t>457677</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>

<commit_message>
Generate .gifs on polyhedron
</commit_message>
<xml_diff>
--- a/system_analysis_overview.xlsx
+++ b/system_analysis_overview.xlsx
@@ -28,25 +28,25 @@
     <t>In-In</t>
   </si>
   <si>
+    <t>451606</t>
+  </si>
+  <si>
+    <t>1410412</t>
+  </si>
+  <si>
+    <t>451623</t>
+  </si>
+  <si>
+    <t>1300872</t>
+  </si>
+  <si>
+    <t>450249</t>
+  </si>
+  <si>
+    <t>1538436</t>
+  </si>
+  <si>
     <t>457677</t>
-  </si>
-  <si>
-    <t>451623</t>
-  </si>
-  <si>
-    <t>1300872</t>
-  </si>
-  <si>
-    <t>1410412</t>
-  </si>
-  <si>
-    <t>450249</t>
-  </si>
-  <si>
-    <t>1538436</t>
-  </si>
-  <si>
-    <t>451606</t>
   </si>
   <si>
     <t>Total</t>

</xml_diff>